<commit_message>
chore: auto sync cms and products backup
</commit_message>
<xml_diff>
--- a/database/CMS_Produk_MitraAbadi_Update.xlsx
+++ b/database/CMS_Produk_MitraAbadi_Update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025\PT MASFOOD WEB\mitra-abadi\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9722DA8E-46DC-4959-8599-714A563A6DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04215041-D458-42AA-BA16-F57B9057EAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2476,7 +2476,8 @@
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30.375" customWidth="1"/>
-    <col min="6" max="6" width="54.75" customWidth="1"/>
+    <col min="6" max="6" width="67" customWidth="1"/>
+    <col min="7" max="7" width="90.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: implement brand logo click filter to product page
</commit_message>
<xml_diff>
--- a/database/CMS_Produk_MitraAbadi_Update.xlsx
+++ b/database/CMS_Produk_MitraAbadi_Update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025\PT MASFOOD WEB\mitra-abadi\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B5B9D3-D358-4EA1-87E9-E3E939251F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE3A2FB-6E6C-460C-BB20-D94F9A8017ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2445" uniqueCount="698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2447" uniqueCount="700">
   <si>
     <t>ID</t>
   </si>
@@ -2114,6 +2114,12 @@
   </si>
   <si>
     <t>Potato Crisps Wavy Mexican Hot Sauce Cans 110g</t>
+  </si>
+  <si>
+    <t>assets/images/products/jacker/hot-spicy-flavor-potato-chips60gr.png</t>
+  </si>
+  <si>
+    <t>assets/images/products/jacker/barbecue-flavor-potato-chips60gr.png</t>
   </si>
 </sst>
 </file>
@@ -2129,7 +2135,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2151,6 +2157,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2182,13 +2194,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3626,7 +3639,7 @@
       <c r="A32" s="1">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="6" t="s">
         <v>678</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -3638,7 +3651,9 @@
       <c r="E32" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F32" s="2"/>
+      <c r="F32" s="3" t="s">
+        <v>698</v>
+      </c>
       <c r="G32" s="1" t="s">
         <v>91</v>
       </c>
@@ -3659,7 +3674,7 @@
       <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="6" t="s">
         <v>677</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -3671,7 +3686,9 @@
       <c r="E33" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F33" s="2"/>
+      <c r="F33" s="2" t="s">
+        <v>699</v>
+      </c>
       <c r="G33" s="1" t="s">
         <v>93</v>
       </c>
@@ -3692,7 +3709,7 @@
       <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="6" t="s">
         <v>94</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -3727,7 +3744,7 @@
       <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="6" t="s">
         <v>679</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -11112,7 +11129,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K1 A7:K17 A6 C6:E6 A5 C5:E5 G5:K5 G6:K6 A100:K100 A99:E99 G99:H99 A102:K105 A101:E101 G101:K101 A98:E98 G98:H98 J98:K98 J99:K99 A107:K108 A106 C106:K106 A110:K130 A109 C109:K109 A132:E132 A131 C131:K131 A135:K165 A133:E133 G133:K133 G132:K132 A134:E134 G134:K134 A34:E34 A31 J31:K31 G31:H31 C31:E31 A196:K245 A195:E195 G195:K195 A181:K194 A180:E180 G180:K180 A167:K179 A166:E166 G166:K166 A32 C32:E32 G32:K32 A33 C33:E33 A36:K97 A35 C35:E35 A30 C30:E30 G30:K30 G33:K33 G34:K34 G35:K35 A29 A24 C24:K24 A23 A18 C18:K18 A19 C19:K19 A20 C20:K20 A21 C21:K21 A22 C22:K22 C23:K23 A25 C25:K25 A26 C26:K26 A27 C27:K27 A28 C28:K28 C29:K29 A3:K4 A2 C2:K2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K1 A7:K17 A6 C6:E6 A5 C5:E5 G5:K5 G6:K6 A100:K100 A99:E99 G99:H99 A102:K105 A101:E101 G101:K101 A98:E98 G98:H98 J98:K98 J99:K99 A107:K108 A106 C106:K106 A110:K130 A109 C109:K109 A132:E132 A131 C131:K131 A135:K165 A133:E133 G133:K133 G132:K132 A134:E134 G134:K134 A34:E34 A31 J31:K31 G31:H31 C31:E31 A196:K245 A195:E195 G195:K195 A181:K194 A180:E180 G180:K180 A167:K179 A166:E166 G166:K166 A32 C32:E32 G32:K32 A33 C33:E33 A36:K97 A35 C35:E35 A30 C30:E30 G30:K30 G33:K33 G34:K34 G35:K35 A29 A24 C24:K24 A23 A18 C18:K18 A19 C19:K19 A20 C20:K20 A21 C21:K21 A22 C22:K22 C23:K23 A25 C25:K25 A26 C26:E26 A27 C27:K27 A28 C28:K28 C29:K29 A3:K4 A2 C2:K2 G26:K26" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>